<commit_message>
refactor: eliminar campo sells_by_weight, derivar de unit como property
</commit_message>
<xml_diff>
--- a/static/templates/SmartVenta_plantilla_importacion_productos.xlsx
+++ b/static/templates/SmartVenta_plantilla_importacion_productos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Reporte" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="24">
   <si>
     <t xml:space="preserve">Código</t>
   </si>
@@ -50,6 +50,9 @@
     <t xml:space="preserve">Precio Mayoreo en descuento de clientes</t>
   </si>
   <si>
+    <t xml:space="preserve">Unidad</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cantidad</t>
   </si>
   <si>
@@ -59,6 +62,9 @@
     <t xml:space="preserve">Opcional</t>
   </si>
   <si>
+    <t xml:space="preserve">PZ|KG|CO</t>
+  </si>
+  <si>
     <t xml:space="preserve">1</t>
   </si>
   <si>
@@ -78,6 +84,9 @@
   </si>
   <si>
     <t xml:space="preserve">Si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PZ</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
@@ -185,7 +194,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -204,6 +213,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -227,8 +240,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultColWidth="8.58984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="8.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.94"/>
@@ -271,6 +284,9 @@
       <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I2" s="3"/>
@@ -278,15 +294,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I4" s="3"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I6" s="5"/>
+      <c r="I6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I7" s="5"/>
+      <c r="I7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I8" s="3"/>
@@ -301,10 +318,10 @@
       <c r="I11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="5"/>
+      <c r="I12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I13" s="5"/>
+      <c r="I13" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -322,7 +339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.22"/>
@@ -334,6 +351,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="38.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -367,86 +385,95 @@
       <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E3" s="0" t="n">
         <v>8</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H3" s="0" t="n">
         <v>5</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E4" s="0" t="n">
         <v>8</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I4" s="3"/>
     </row>

</xml_diff>